<commit_message>
feat(calculators): first test case for 3.4 method 1 passing
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.4-sheep-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.4-sheep-enteric.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{7D182355-8DF9-5648-A887-8B96E1FF671F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{1D753D7A-07C6-4342-9D2D-5A7E28B713C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="1600" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3.4.1.1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="98">
   <si>
     <t>(LRjk=3,4 * min( LMRjk=3,4  100)) / 100</t>
   </si>
@@ -319,6 +319,15 @@
   </si>
   <si>
     <t>A.1.4.1</t>
+  </si>
+  <si>
+    <t>Custom Wjk</t>
+  </si>
+  <si>
+    <t>Custom DMA</t>
+  </si>
+  <si>
+    <t>Custom DMD</t>
   </si>
 </sst>
 </file>
@@ -334,12 +343,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -354,8 +375,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,36 +713,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:AE95"/>
+  <dimension ref="A2:AH95"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.2">
       <c r="G2" t="s">
         <v>0</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>1</v>
       </c>
-      <c r="M2" t="s">
+      <c r="P2" t="s">
         <v>2</v>
       </c>
-      <c r="N2" t="s">
+      <c r="Q2" t="s">
         <v>3</v>
       </c>
-      <c r="O2" t="s">
+      <c r="R2" t="s">
         <v>4</v>
       </c>
-      <c r="P2" t="s">
+      <c r="S2" t="s">
         <v>5</v>
       </c>
-      <c r="R2" t="s">
+      <c r="U2" t="s">
         <v>6</v>
       </c>
-      <c r="T2" t="s">
+      <c r="W2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
       <c r="E3" t="s">
         <v>8</v>
       </c>
@@ -732,53 +755,53 @@
       <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>12</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>13</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>14</v>
       </c>
-      <c r="L3" t="s">
+      <c r="O3" t="s">
         <v>15</v>
       </c>
-      <c r="M3" t="s">
+      <c r="P3" t="s">
         <v>16</v>
       </c>
-      <c r="N3" t="s">
+      <c r="Q3" t="s">
         <v>17</v>
       </c>
-      <c r="O3" t="s">
+      <c r="R3" t="s">
         <v>18</v>
       </c>
-      <c r="P3" t="s">
+      <c r="S3" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="T3" t="s">
         <v>20</v>
       </c>
-      <c r="R3" t="s">
+      <c r="U3" t="s">
         <v>21</v>
       </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>22</v>
       </c>
-      <c r="T3" t="s">
+      <c r="W3" t="s">
         <v>23</v>
       </c>
-      <c r="X3">
+      <c r="AA3">
         <v>351</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="AB3" t="s">
         <v>57</v>
       </c>
-      <c r="Z3">
+      <c r="AC3">
         <v>1.3</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
       <c r="E4" t="s">
         <v>24</v>
       </c>
@@ -791,44 +814,53 @@
       <c r="H4" t="s">
         <v>26</v>
       </c>
-      <c r="I4" t="s">
-        <v>26</v>
-      </c>
       <c r="J4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" t="s">
-        <v>25</v>
-      </c>
       <c r="L4" t="s">
         <v>26</v>
       </c>
       <c r="M4" t="s">
         <v>25</v>
       </c>
-      <c r="N4" t="s">
-        <v>25</v>
-      </c>
       <c r="O4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P4" t="s">
         <v>25</v>
       </c>
       <c r="Q4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R4" t="s">
         <v>25</v>
       </c>
       <c r="S4" t="s">
+        <v>25</v>
+      </c>
+      <c r="T4" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" t="s">
         <v>26</v>
       </c>
-      <c r="T4" t="s">
+      <c r="W4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AA4">
+        <v>346</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AC4">
+        <v>91.25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
       <c r="E5" t="s">
         <v>27</v>
       </c>
@@ -841,26 +873,17 @@
       <c r="H5" t="s">
         <v>27</v>
       </c>
-      <c r="I5" t="s">
-        <v>24</v>
-      </c>
       <c r="J5" t="s">
         <v>24</v>
       </c>
-      <c r="K5" t="s">
-        <v>27</v>
-      </c>
       <c r="L5" t="s">
         <v>24</v>
       </c>
       <c r="M5" t="s">
         <v>27</v>
       </c>
-      <c r="N5" t="s">
-        <v>27</v>
-      </c>
       <c r="O5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="P5" t="s">
         <v>27</v>
@@ -872,13 +895,22 @@
         <v>27</v>
       </c>
       <c r="S5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="T5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="U5" t="s">
+        <v>27</v>
+      </c>
+      <c r="V5" t="s">
+        <v>24</v>
+      </c>
+      <c r="W5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
       <c r="E8" t="s">
         <v>28</v>
       </c>
@@ -891,44 +923,47 @@
       <c r="H8" t="s">
         <v>29</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>30</v>
       </c>
-      <c r="J8" t="s">
+      <c r="L8" t="s">
         <v>28</v>
       </c>
-      <c r="K8" t="s">
+      <c r="M8" t="s">
         <v>31</v>
       </c>
-      <c r="L8" t="s">
+      <c r="O8" t="s">
         <v>32</v>
-      </c>
-      <c r="M8" t="s">
-        <v>33</v>
-      </c>
-      <c r="N8" t="s">
-        <v>31</v>
-      </c>
-      <c r="O8" t="s">
-        <v>31</v>
       </c>
       <c r="P8" t="s">
         <v>33</v>
       </c>
       <c r="Q8" t="s">
+        <v>31</v>
+      </c>
+      <c r="R8" t="s">
+        <v>31</v>
+      </c>
+      <c r="S8" t="s">
+        <v>33</v>
+      </c>
+      <c r="T8" t="s">
         <v>34</v>
       </c>
-      <c r="R8" t="s">
+      <c r="U8" t="s">
         <v>35</v>
       </c>
-      <c r="S8" t="s">
+      <c r="V8" t="s">
         <v>36</v>
       </c>
-      <c r="T8" t="s">
+      <c r="W8" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="X8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
       <c r="E9" t="s">
         <v>38</v>
       </c>
@@ -941,44 +976,44 @@
       <c r="H9" t="s">
         <v>41</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>42</v>
       </c>
-      <c r="J9" t="s">
+      <c r="L9" t="s">
         <v>43</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>44</v>
       </c>
-      <c r="L9" t="s">
+      <c r="O9" t="s">
         <v>45</v>
       </c>
-      <c r="M9" t="s">
+      <c r="P9" t="s">
         <v>46</v>
       </c>
-      <c r="N9" t="s">
+      <c r="Q9" t="s">
         <v>47</v>
       </c>
-      <c r="O9" t="s">
+      <c r="R9" t="s">
         <v>48</v>
       </c>
-      <c r="P9" t="s">
+      <c r="S9" t="s">
         <v>49</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="T9" t="s">
         <v>50</v>
       </c>
-      <c r="R9" t="s">
+      <c r="U9" t="s">
         <v>51</v>
       </c>
-      <c r="S9" t="s">
+      <c r="V9" t="s">
         <v>52</v>
       </c>
-      <c r="T9" t="s">
+      <c r="W9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>70</v>
       </c>
@@ -991,10 +1026,10 @@
       <c r="D10" t="s">
         <v>79</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>55</v>
       </c>
       <c r="G10" t="s">
@@ -1004,43 +1039,55 @@
         <v>57</v>
       </c>
       <c r="I10" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" t="s">
         <v>58</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" t="s">
         <v>59</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M10" t="s">
         <v>60</v>
       </c>
-      <c r="L10" t="s">
+      <c r="N10" t="s">
+        <v>95</v>
+      </c>
+      <c r="O10" t="s">
         <v>61</v>
       </c>
-      <c r="M10" t="s">
+      <c r="P10" t="s">
         <v>62</v>
       </c>
-      <c r="N10" t="s">
+      <c r="Q10" t="s">
         <v>63</v>
       </c>
-      <c r="O10" t="s">
+      <c r="R10" t="s">
         <v>64</v>
       </c>
-      <c r="P10" t="s">
+      <c r="S10" t="s">
         <v>65</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="T10" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="R10" t="s">
+      <c r="U10" t="s">
         <v>67</v>
       </c>
-      <c r="S10" t="s">
+      <c r="V10" t="s">
         <v>68</v>
       </c>
-      <c r="T10" t="s">
+      <c r="W10" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="X10" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -1062,44 +1109,58 @@
       <c r="G11">
         <v>0</v>
       </c>
-      <c r="I11">
-        <f>$Z$17</f>
+      <c r="J11">
+        <f>$AC$17</f>
         <v>2.9</v>
       </c>
-      <c r="J11">
-        <f>$Z$45</f>
+      <c r="L11">
+        <f>$AC$45</f>
         <v>0.75</v>
       </c>
-      <c r="K11">
-        <f>(0.795 * J11) - 0.0014</f>
+      <c r="M11">
+        <f>(0.795 * L11) - 0.0014</f>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L11">
-        <f>$Z72</f>
+      <c r="O11">
+        <f>$AC72</f>
         <v>75</v>
       </c>
-      <c r="M11">
-        <f>(104.7 * K11 + 0.307 * L11- 15) * L11 * 10^-3</f>
-        <v>5.2729346250000022</v>
-      </c>
-      <c r="N11">
-        <f>1-EXP(-2*POWER(I11,2))</f>
+      <c r="P11">
+        <f>(104.7 * M11 + 0.307 * O11- 15) * POWER(O11, 0.75) * 10^-3</f>
+        <v>1.7917898456122741</v>
+      </c>
+      <c r="Q11">
+        <f>1-EXP(-2*POWER(J11,2))</f>
         <v>0.9999999504359468</v>
       </c>
-      <c r="O11">
-        <f>(G11 * H11) + (1 - G11)</f>
+      <c r="R11">
         <v>1</v>
       </c>
-      <c r="P11">
-        <f>M11 * N11 * O11</f>
-        <v>5.2729343636519896</v>
-      </c>
-      <c r="R11">
-        <f>(P11 * 0.0188) + 0.00158</f>
-        <v>0.1007111660366574</v>
-      </c>
-    </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="S11">
+        <f>P11 * Q11 * R11</f>
+        <v>1.7917897568039067</v>
+      </c>
+      <c r="T11">
+        <v>50</v>
+      </c>
+      <c r="U11">
+        <f>(S11 * 0.0188) + 0.00158</f>
+        <v>3.5265647427913445E-2</v>
+      </c>
+      <c r="V11">
+        <f>$AC$4</f>
+        <v>91.25</v>
+      </c>
+      <c r="W11">
+        <f>T11*U11*V11</f>
+        <v>160.89951638985508</v>
+      </c>
+      <c r="X11">
+        <f>SUM(W11:W34)*10^-3</f>
+        <v>3.7707328300265006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
         <v>81</v>
       </c>
@@ -1112,32 +1173,54 @@
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="I12">
-        <f>$Z$18</f>
+      <c r="J12">
+        <f>$AC$18</f>
         <v>2.5</v>
       </c>
-      <c r="J12">
-        <f>$Z$46</f>
+      <c r="L12">
+        <f>$AC$46</f>
         <v>0.61</v>
       </c>
-      <c r="K12">
-        <f t="shared" ref="K12:K34" si="0">(0.795 * J12) - 0.0014</f>
+      <c r="M12">
+        <f t="shared" ref="M12:M34" si="0">(0.795 * L12) - 0.0014</f>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L12">
-        <f t="shared" ref="L12:L14" si="1">$Z73</f>
+      <c r="O12">
+        <f t="shared" ref="O12:O14" si="1">$AC73</f>
         <v>75</v>
       </c>
-      <c r="M12">
-        <f t="shared" ref="M12:M33" si="2">(104.7 * K12 + 0.307 * L12- 15) * L12 * 10^-3</f>
-        <v>4.3989513749999993</v>
-      </c>
-      <c r="N12">
-        <f t="shared" ref="N12:N34" si="3">1-EXP(-2*POWER(I12,2))</f>
+      <c r="P12">
+        <f>(104.7 * M12 + 0.307 * O12- 15) * POWER(O12, 0.75) * 10^-3</f>
+        <v>1.4948026034112167</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" ref="Q12:Q34" si="2">1-EXP(-2*POWER(J12,2))</f>
         <v>0.99999627334682795</v>
       </c>
-    </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12">
+        <f t="shared" ref="S12:S34" si="3">P12 * Q12 * R12</f>
+        <v>1.494797032800353</v>
+      </c>
+      <c r="T12">
+        <v>40</v>
+      </c>
+      <c r="U12">
+        <f t="shared" ref="U12:U34" si="4">(S12 * 0.0188) + 0.00158</f>
+        <v>2.9682184216646638E-2</v>
+      </c>
+      <c r="V12">
+        <f t="shared" ref="V12:V34" si="5">$AC$4</f>
+        <v>91.25</v>
+      </c>
+      <c r="W12">
+        <f t="shared" ref="W12:W34" si="6">T12*U12*V12</f>
+        <v>108.33997239076024</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D13" t="s">
         <v>82</v>
       </c>
@@ -1150,32 +1233,54 @@
       <c r="G13">
         <v>0</v>
       </c>
-      <c r="I13">
-        <f>$Z$19</f>
+      <c r="J13">
+        <f>$AC$19</f>
         <v>1.6</v>
       </c>
-      <c r="J13">
-        <f>$Z$47</f>
+      <c r="L13">
+        <f>$AC$47</f>
         <v>0.64</v>
       </c>
-      <c r="K13">
+      <c r="M13">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L13">
+      <c r="O13">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="M13">
+      <c r="P13">
+        <f t="shared" ref="P13:P34" si="7">(104.7 * M13 + 0.307 * O13- 15) * POWER(O13, 0.75) * 10^-3</f>
+        <v>1.4198696820048529</v>
+      </c>
+      <c r="Q13">
         <f t="shared" si="2"/>
-        <v>4.092236820000001</v>
-      </c>
-      <c r="N13">
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13">
         <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-    </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.2">
+        <v>1.4113845082772669</v>
+      </c>
+      <c r="T13">
+        <v>38</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="4"/>
+        <v>2.811402875561262E-2</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="6"/>
+        <v>97.485394710086752</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D14" t="s">
         <v>83</v>
       </c>
@@ -1188,35 +1293,57 @@
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="I14">
-        <f>$Z$20</f>
+      <c r="J14">
+        <f>$AC$20</f>
         <v>1.7</v>
       </c>
-      <c r="J14">
-        <f>$Z$48</f>
+      <c r="L14">
+        <f>$AC$48</f>
         <v>0.72</v>
       </c>
-      <c r="K14">
+      <c r="M14">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L14">
+      <c r="O14">
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="M14">
+      <c r="P14">
+        <f t="shared" si="7"/>
+        <v>1.5792888783210146</v>
+      </c>
+      <c r="Q14">
         <f t="shared" si="2"/>
-        <v>4.5517022999999996</v>
-      </c>
-      <c r="N14">
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14">
         <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y14" t="s">
+        <v>1.5744109044284875</v>
+      </c>
+      <c r="T14">
+        <v>50</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="4"/>
+        <v>3.1178925003255569E-2</v>
+      </c>
+      <c r="V14">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W14">
+        <f t="shared" si="6"/>
+        <v>142.25384532735353</v>
+      </c>
+      <c r="AB14" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1235,35 +1362,57 @@
       <c r="G15">
         <v>0</v>
       </c>
-      <c r="I15">
-        <f>$AA$17</f>
+      <c r="J15">
+        <f>$AD$17</f>
         <v>2.9</v>
       </c>
-      <c r="J15">
-        <f>$AA$45</f>
+      <c r="L15">
+        <f>$AD$45</f>
         <v>0.75</v>
       </c>
-      <c r="K15">
+      <c r="M15">
         <f t="shared" si="0"/>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L15">
-        <f>$AA72</f>
+      <c r="O15">
+        <f>$AD72</f>
         <v>62</v>
       </c>
-      <c r="M15">
+      <c r="P15">
+        <f t="shared" si="7"/>
+        <v>1.4652245899459331</v>
+      </c>
+      <c r="Q15">
         <f t="shared" si="2"/>
-        <v>4.1115172900000001</v>
-      </c>
-      <c r="N15">
+        <v>0.9999999504359468</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15">
         <f t="shared" si="3"/>
-        <v>0.9999999504359468</v>
-      </c>
-      <c r="Y15" t="s">
+        <v>1.4652245173234635</v>
+      </c>
+      <c r="T15">
+        <v>100</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="4"/>
+        <v>2.9126220925681116E-2</v>
+      </c>
+      <c r="V15">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W15">
+        <f t="shared" si="6"/>
+        <v>265.77676594684021</v>
+      </c>
+      <c r="AB15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
         <v>81</v>
       </c>
@@ -1276,50 +1425,72 @@
       <c r="G16">
         <v>0</v>
       </c>
-      <c r="I16">
-        <f>$AA$18</f>
+      <c r="J16">
+        <f>$AD$18</f>
         <v>2.5</v>
       </c>
-      <c r="J16">
-        <f>$AA$46</f>
+      <c r="L16">
+        <f>$AD$46</f>
         <v>0.61</v>
       </c>
-      <c r="K16">
+      <c r="M16">
         <f t="shared" si="0"/>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L16">
-        <f t="shared" ref="L16:L18" si="4">$AA73</f>
+      <c r="O16">
+        <f t="shared" ref="O16:O18" si="8">$AD73</f>
         <v>55</v>
       </c>
-      <c r="M16">
+      <c r="P16">
+        <f t="shared" si="7"/>
+        <v>1.0605624381175847</v>
+      </c>
+      <c r="Q16">
         <f t="shared" si="2"/>
-        <v>2.8881976750000002</v>
-      </c>
-      <c r="N16">
+        <v>0.99999627334682795</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16">
         <f t="shared" si="3"/>
-        <v>0.99999627334682795</v>
-      </c>
-      <c r="Z16" t="s">
+        <v>1.0605584857692105</v>
+      </c>
+      <c r="T16">
+        <v>120</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="4"/>
+        <v>2.1518499532461158E-2</v>
+      </c>
+      <c r="V16">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W16">
+        <f t="shared" si="6"/>
+        <v>235.6275698804497</v>
+      </c>
+      <c r="AC16" t="s">
         <v>72</v>
       </c>
-      <c r="AA16" t="s">
+      <c r="AD16" t="s">
         <v>73</v>
       </c>
-      <c r="AB16" t="s">
+      <c r="AE16" t="s">
         <v>74</v>
       </c>
-      <c r="AC16" t="s">
+      <c r="AF16" t="s">
         <v>75</v>
       </c>
-      <c r="AD16" t="s">
+      <c r="AG16" t="s">
         <v>76</v>
       </c>
-      <c r="AE16" t="s">
+      <c r="AH16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D17" t="s">
         <v>82</v>
       </c>
@@ -1332,44 +1503,57 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="I17">
-        <f>$AA$19</f>
+      <c r="J17">
+        <f>$AD$19</f>
         <v>1.6</v>
       </c>
-      <c r="J17">
-        <f>$AA$47</f>
+      <c r="L17">
+        <f>$AD$47</f>
         <v>0.64</v>
       </c>
-      <c r="K17">
+      <c r="M17">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L17">
+      <c r="O17">
+        <f t="shared" si="8"/>
+        <v>55</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="7"/>
+        <v>1.1109945415495692</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="2"/>
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R17">
+        <v>1</v>
+      </c>
+      <c r="S17">
+        <f t="shared" si="3"/>
+        <v>1.1043552127330423</v>
+      </c>
+      <c r="T17">
+        <v>115</v>
+      </c>
+      <c r="U17">
         <f t="shared" si="4"/>
-        <v>55</v>
-      </c>
-      <c r="M17">
-        <f t="shared" si="2"/>
-        <v>3.0255379000000002</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-      <c r="X17" t="s">
+        <v>2.2341877999381195E-2</v>
+      </c>
+      <c r="V17">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W17">
+        <f t="shared" si="6"/>
+        <v>234.4500822560064</v>
+      </c>
+      <c r="AA17" t="s">
         <v>85</v>
       </c>
-      <c r="Y17" t="s">
+      <c r="AB17" t="s">
         <v>80</v>
-      </c>
-      <c r="Z17">
-        <v>2.9</v>
-      </c>
-      <c r="AA17">
-        <v>2.9</v>
-      </c>
-      <c r="AB17">
-        <v>2.9</v>
       </c>
       <c r="AC17">
         <v>2.9</v>
@@ -1380,8 +1564,17 @@
       <c r="AE17">
         <v>2.9</v>
       </c>
-    </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF17">
+        <v>2.9</v>
+      </c>
+      <c r="AG17">
+        <v>2.9</v>
+      </c>
+      <c r="AH17">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D18" t="s">
         <v>83</v>
       </c>
@@ -1394,41 +1587,54 @@
       <c r="G18">
         <v>0</v>
       </c>
-      <c r="I18">
-        <f>$AA$20</f>
+      <c r="J18">
+        <f>$AD$20</f>
         <v>1.7</v>
       </c>
-      <c r="J18">
-        <f>$AA$48</f>
+      <c r="L18">
+        <f>$AD$48</f>
         <v>0.72</v>
       </c>
-      <c r="K18">
+      <c r="M18">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L18">
+      <c r="O18">
+        <f t="shared" si="8"/>
+        <v>55</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="7"/>
+        <v>1.2454801507015281</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="2"/>
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R18">
+        <v>1</v>
+      </c>
+      <c r="S18">
+        <f t="shared" si="3"/>
+        <v>1.2416332169694033</v>
+      </c>
+      <c r="T18">
+        <v>110</v>
+      </c>
+      <c r="U18">
         <f t="shared" si="4"/>
-        <v>55</v>
-      </c>
-      <c r="M18">
-        <f t="shared" si="2"/>
-        <v>3.3917785</v>
-      </c>
-      <c r="N18">
-        <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y18" t="s">
+        <v>2.4922704479024786E-2</v>
+      </c>
+      <c r="V18">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W18">
+        <f t="shared" si="6"/>
+        <v>250.16164620821129</v>
+      </c>
+      <c r="AB18" t="s">
         <v>81</v>
-      </c>
-      <c r="Z18">
-        <v>2.5</v>
-      </c>
-      <c r="AA18">
-        <v>2.5</v>
-      </c>
-      <c r="AB18">
-        <v>2.5</v>
       </c>
       <c r="AC18">
         <v>2.5</v>
@@ -1439,8 +1645,17 @@
       <c r="AE18">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF18">
+        <v>2.5</v>
+      </c>
+      <c r="AG18">
+        <v>2.5</v>
+      </c>
+      <c r="AH18">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>3</v>
       </c>
@@ -1457,48 +1672,62 @@
         <v>85</v>
       </c>
       <c r="G19">
-        <f>(E19*MIN(F19,100))/100</f>
-        <v>76.5</v>
+        <f>(E19/100*MIN(F19,100)/100)</f>
+        <v>0.76500000000000001</v>
       </c>
       <c r="H19">
-        <f>$Z$3</f>
+        <f>$AC$3</f>
         <v>1.3</v>
       </c>
-      <c r="I19">
-        <f>$AB$17</f>
+      <c r="J19">
+        <f>$AE$17</f>
         <v>2.9</v>
       </c>
-      <c r="J19">
-        <f>$AB$45</f>
+      <c r="L19">
+        <f>$AE$45</f>
         <v>0.75</v>
       </c>
-      <c r="K19">
+      <c r="M19">
         <f t="shared" si="0"/>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L19">
-        <f>$AB72</f>
+      <c r="O19">
+        <f>$AE72</f>
         <v>44</v>
       </c>
-      <c r="M19">
+      <c r="P19">
+        <f>(104.7 * M19 + 0.307 * O19- 15) * POWER(O19, 0.75) * 10^-3</f>
+        <v>1.0385156413271623</v>
+      </c>
+      <c r="Q19">
         <f t="shared" si="2"/>
-        <v>2.6747069800000003</v>
-      </c>
-      <c r="N19">
+        <v>0.9999999504359468</v>
+      </c>
+      <c r="R19">
+        <f>(G19 * H19) + (1 - G19)</f>
+        <v>1.2295</v>
+      </c>
+      <c r="S19">
         <f t="shared" si="3"/>
-        <v>0.9999999504359468</v>
-      </c>
-      <c r="Y19" t="s">
+        <v>1.2768549177256379</v>
+      </c>
+      <c r="T19">
+        <v>120</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="4"/>
+        <v>2.5584872453241994E-2</v>
+      </c>
+      <c r="V19">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W19">
+        <f t="shared" si="6"/>
+        <v>280.15435336299987</v>
+      </c>
+      <c r="AB19" t="s">
         <v>82</v>
-      </c>
-      <c r="Z19">
-        <v>1.6</v>
-      </c>
-      <c r="AA19">
-        <v>1.6</v>
-      </c>
-      <c r="AB19">
-        <v>1.6</v>
       </c>
       <c r="AC19">
         <v>1.6</v>
@@ -1509,8 +1738,17 @@
       <c r="AE19">
         <v>1.6</v>
       </c>
-    </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF19">
+        <v>1.6</v>
+      </c>
+      <c r="AG19">
+        <v>1.6</v>
+      </c>
+      <c r="AH19">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
         <v>81</v>
       </c>
@@ -1521,43 +1759,58 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <f>$AB$18</f>
+        <f>(E20/100*MIN(F20,100)/100)</f>
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <f>$AE$18</f>
         <v>2.5</v>
       </c>
-      <c r="J20">
-        <f>$AB$46</f>
+      <c r="L20">
+        <f>$AE$46</f>
         <v>0.61</v>
       </c>
-      <c r="K20">
+      <c r="M20">
         <f t="shared" si="0"/>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L20">
-        <f t="shared" ref="L20:L22" si="5">$AB73</f>
+      <c r="O20">
+        <f t="shared" ref="O20:O22" si="9">$AE73</f>
         <v>42</v>
       </c>
-      <c r="M20">
+      <c r="P20">
+        <f t="shared" si="7"/>
+        <v>0.80052120768394575</v>
+      </c>
+      <c r="Q20">
         <f t="shared" si="2"/>
-        <v>2.0379107699999999</v>
-      </c>
-      <c r="N20">
+        <v>0.99999627334682795</v>
+      </c>
+      <c r="R20">
+        <f t="shared" ref="R20:R26" si="10">(G20 * H20) + (1 - G20)</f>
+        <v>1</v>
+      </c>
+      <c r="S20">
         <f t="shared" si="3"/>
-        <v>0.99999627334682795</v>
-      </c>
-      <c r="Y20" t="s">
+        <v>0.80051822441904785</v>
+      </c>
+      <c r="T20">
+        <v>130</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="4"/>
+        <v>1.6629742619078101E-2</v>
+      </c>
+      <c r="V20">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W20">
+        <f t="shared" si="6"/>
+        <v>197.27032181881395</v>
+      </c>
+      <c r="AB20" t="s">
         <v>83</v>
-      </c>
-      <c r="Z20">
-        <v>1.7</v>
-      </c>
-      <c r="AA20">
-        <v>1.7</v>
-      </c>
-      <c r="AB20">
-        <v>1.7</v>
       </c>
       <c r="AC20">
         <v>1.7</v>
@@ -1568,8 +1821,17 @@
       <c r="AE20">
         <v>1.7</v>
       </c>
-    </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF20">
+        <v>1.7</v>
+      </c>
+      <c r="AG20">
+        <v>1.7</v>
+      </c>
+      <c r="AH20">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D21" t="s">
         <v>82</v>
       </c>
@@ -1580,46 +1842,61 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="I21">
-        <f>$AB$19</f>
+        <f t="shared" ref="G21:G23" si="11">(E21/100*MIN(F21,100)/100)</f>
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <f>$AE$19</f>
         <v>1.6</v>
       </c>
-      <c r="J21">
-        <f>$AB$47</f>
+      <c r="L21">
+        <f>$AE$47</f>
         <v>0.64</v>
       </c>
-      <c r="K21">
+      <c r="M21">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L21">
+      <c r="O21">
+        <f t="shared" si="9"/>
+        <v>43</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="7"/>
+        <v>0.86186034677094148</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="2"/>
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="S21">
+        <f t="shared" si="3"/>
+        <v>0.85670984960634056</v>
+      </c>
+      <c r="T21">
+        <v>120</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="4"/>
+        <v>1.7686145172599206E-2</v>
+      </c>
+      <c r="V21">
         <f t="shared" si="5"/>
-        <v>43</v>
-      </c>
-      <c r="M21">
-        <f t="shared" si="2"/>
-        <v>2.2070085400000004</v>
-      </c>
-      <c r="N21">
-        <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-      <c r="X21" t="s">
+        <v>91.25</v>
+      </c>
+      <c r="W21">
+        <f t="shared" si="6"/>
+        <v>193.66328963996131</v>
+      </c>
+      <c r="AA21" t="s">
         <v>86</v>
       </c>
-      <c r="Y21" t="s">
+      <c r="AB21" t="s">
         <v>80</v>
-      </c>
-      <c r="Z21">
-        <v>1.5</v>
-      </c>
-      <c r="AA21">
-        <v>1.5</v>
-      </c>
-      <c r="AB21">
-        <v>1.5</v>
       </c>
       <c r="AC21">
         <v>1.5</v>
@@ -1630,8 +1907,17 @@
       <c r="AE21">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF21">
+        <v>1.5</v>
+      </c>
+      <c r="AG21">
+        <v>1.5</v>
+      </c>
+      <c r="AH21">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D22" t="s">
         <v>83</v>
       </c>
@@ -1642,43 +1928,58 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="I22">
-        <f>$AB$20</f>
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <f>$AE$20</f>
         <v>1.7</v>
       </c>
-      <c r="J22">
-        <f>$AB$48</f>
+      <c r="L22">
+        <f>$AE$48</f>
         <v>0.72</v>
       </c>
-      <c r="K22">
+      <c r="M22">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L22">
+      <c r="O22">
+        <f t="shared" si="9"/>
+        <v>45</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="7"/>
+        <v>1.0181162441707754</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="2"/>
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="S22">
+        <f t="shared" si="3"/>
+        <v>1.014971572840029</v>
+      </c>
+      <c r="T22">
+        <v>110</v>
+      </c>
+      <c r="U22">
+        <f t="shared" si="4"/>
+        <v>2.0661465569392547E-2</v>
+      </c>
+      <c r="V22">
         <f t="shared" si="5"/>
-        <v>45</v>
-      </c>
-      <c r="M22">
-        <f t="shared" si="2"/>
-        <v>2.6369415000000003</v>
-      </c>
-      <c r="N22">
-        <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y22" t="s">
+        <v>91.25</v>
+      </c>
+      <c r="W22">
+        <f t="shared" si="6"/>
+        <v>207.3894606527777</v>
+      </c>
+      <c r="AB22" t="s">
         <v>81</v>
-      </c>
-      <c r="Z22">
-        <v>2</v>
-      </c>
-      <c r="AA22">
-        <v>2</v>
-      </c>
-      <c r="AB22">
-        <v>2</v>
       </c>
       <c r="AC22">
         <v>2</v>
@@ -1689,8 +1990,17 @@
       <c r="AE22">
         <v>2</v>
       </c>
-    </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF22">
+        <v>2</v>
+      </c>
+      <c r="AG22">
+        <v>2</v>
+      </c>
+      <c r="AH22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4</v>
       </c>
@@ -1707,48 +2017,62 @@
         <v>88</v>
       </c>
       <c r="G23">
-        <f>(E23*MIN(F23,100))/100</f>
-        <v>83.6</v>
+        <f t="shared" si="11"/>
+        <v>0.83599999999999997</v>
       </c>
       <c r="H23">
-        <f>$Z$3</f>
+        <f>$AC$3</f>
         <v>1.3</v>
       </c>
-      <c r="I23">
-        <f>$AC$17</f>
+      <c r="J23">
+        <f>$AF$17</f>
         <v>2.9</v>
       </c>
-      <c r="J23">
-        <f>$AC$45</f>
+      <c r="L23">
+        <f>$AF$45</f>
         <v>0.75</v>
       </c>
-      <c r="K23">
+      <c r="M23">
         <f t="shared" si="0"/>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L23">
-        <f>$AC72</f>
+      <c r="O23">
+        <f>$AF72</f>
         <v>54</v>
       </c>
-      <c r="M23">
+      <c r="P23">
+        <f t="shared" si="7"/>
+        <v>1.2720847291262878</v>
+      </c>
+      <c r="Q23">
         <f t="shared" si="2"/>
-        <v>3.4483749300000008</v>
-      </c>
-      <c r="N23">
+        <v>0.9999999504359468</v>
+      </c>
+      <c r="R23">
+        <f t="shared" si="10"/>
+        <v>1.2507999999999999</v>
+      </c>
+      <c r="S23">
         <f t="shared" si="3"/>
-        <v>0.9999999504359468</v>
-      </c>
-      <c r="Y23" t="s">
+        <v>1.5911235003286268</v>
+      </c>
+      <c r="T23">
+        <v>80</v>
+      </c>
+      <c r="U23">
+        <f t="shared" si="4"/>
+        <v>3.1493121806178186E-2</v>
+      </c>
+      <c r="V23">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W23">
+        <f t="shared" si="6"/>
+        <v>229.89978918510076</v>
+      </c>
+      <c r="AB23" t="s">
         <v>82</v>
-      </c>
-      <c r="Z23">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="AA23">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="AB23">
-        <v>2.2000000000000002</v>
       </c>
       <c r="AC23">
         <v>2.2000000000000002</v>
@@ -1759,8 +2083,17 @@
       <c r="AE23">
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF23">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AG23">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AH23">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
         <v>81</v>
       </c>
@@ -1773,41 +2106,55 @@
       <c r="G24">
         <v>0</v>
       </c>
-      <c r="I24">
-        <f>$AC$18</f>
+      <c r="J24">
+        <f>$AF$18</f>
         <v>2.5</v>
       </c>
-      <c r="J24">
-        <f>$AC$46</f>
+      <c r="L24">
+        <f>$AF$46</f>
         <v>0.61</v>
       </c>
-      <c r="K24">
+      <c r="M24">
         <f t="shared" si="0"/>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L24">
-        <f t="shared" ref="L24:L26" si="6">$AC73</f>
+      <c r="O24">
+        <f t="shared" ref="O24:O26" si="12">$AF73</f>
         <v>49</v>
       </c>
-      <c r="M24">
+      <c r="P24">
+        <f t="shared" si="7"/>
+        <v>0.93843421889903578</v>
+      </c>
+      <c r="Q24">
         <f t="shared" si="2"/>
-        <v>2.4828635649999997</v>
-      </c>
-      <c r="N24">
+        <v>0.99999627334682795</v>
+      </c>
+      <c r="R24">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="S24">
         <f t="shared" si="3"/>
-        <v>0.99999627334682795</v>
-      </c>
-      <c r="Y24" t="s">
+        <v>0.93843072168017716</v>
+      </c>
+      <c r="T24">
+        <v>90</v>
+      </c>
+      <c r="U24">
+        <f t="shared" si="4"/>
+        <v>1.9222497567587333E-2</v>
+      </c>
+      <c r="V24">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W24">
+        <f t="shared" si="6"/>
+        <v>157.86476127381098</v>
+      </c>
+      <c r="AB24" t="s">
         <v>83</v>
-      </c>
-      <c r="Z24">
-        <v>1.7</v>
-      </c>
-      <c r="AA24">
-        <v>1.7</v>
-      </c>
-      <c r="AB24">
-        <v>1.7</v>
       </c>
       <c r="AC24">
         <v>1.7</v>
@@ -1818,8 +2165,17 @@
       <c r="AE24">
         <v>1.7</v>
       </c>
-    </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF24">
+        <v>1.7</v>
+      </c>
+      <c r="AG24">
+        <v>1.7</v>
+      </c>
+      <c r="AH24">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D25" t="s">
         <v>82</v>
       </c>
@@ -1832,44 +2188,58 @@
       <c r="G25">
         <v>0</v>
       </c>
-      <c r="I25">
-        <f>$AC$19</f>
+      <c r="J25">
+        <f>$AF$19</f>
         <v>1.6</v>
       </c>
-      <c r="J25">
-        <f>$AC$47</f>
+      <c r="L25">
+        <f>$AF$47</f>
         <v>0.64</v>
       </c>
-      <c r="K25">
+      <c r="M25">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L25">
+      <c r="O25">
+        <f t="shared" si="12"/>
+        <v>50</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="7"/>
+        <v>1.0054871153505722</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="2"/>
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R25">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="S25">
+        <f t="shared" si="3"/>
+        <v>0.99947830132860371</v>
+      </c>
+      <c r="T25">
+        <v>80</v>
+      </c>
+      <c r="U25">
+        <f t="shared" si="4"/>
+        <v>2.0370192064977751E-2</v>
+      </c>
+      <c r="V25">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W25">
         <f t="shared" si="6"/>
-        <v>50</v>
-      </c>
-      <c r="M25">
-        <f t="shared" si="2"/>
-        <v>2.6737390000000008</v>
-      </c>
-      <c r="N25">
-        <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-      <c r="X25" t="s">
+        <v>148.70240207433758</v>
+      </c>
+      <c r="AA25" t="s">
         <v>87</v>
       </c>
-      <c r="Y25" t="s">
+      <c r="AB25" t="s">
         <v>80</v>
-      </c>
-      <c r="Z25">
-        <v>4</v>
-      </c>
-      <c r="AA25">
-        <v>4</v>
-      </c>
-      <c r="AB25">
-        <v>4</v>
       </c>
       <c r="AC25">
         <v>4</v>
@@ -1880,8 +2250,17 @@
       <c r="AE25">
         <v>4</v>
       </c>
-    </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF25">
+        <v>4</v>
+      </c>
+      <c r="AG25">
+        <v>4</v>
+      </c>
+      <c r="AH25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D26" t="s">
         <v>83</v>
       </c>
@@ -1894,41 +2273,55 @@
       <c r="G26">
         <v>0</v>
       </c>
-      <c r="I26">
-        <f>$AC$20</f>
+      <c r="J26">
+        <f>$AF$20</f>
         <v>1.7</v>
       </c>
-      <c r="J26">
-        <f>$AC$48</f>
+      <c r="L26">
+        <f>$AF$48</f>
         <v>0.72</v>
       </c>
-      <c r="K26">
+      <c r="M26">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L26">
+      <c r="O26">
+        <f t="shared" si="12"/>
+        <v>50</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="7"/>
+        <v>1.1306948910936463</v>
+      </c>
+      <c r="Q26">
+        <f t="shared" si="2"/>
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R26">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="S26">
+        <f t="shared" si="3"/>
+        <v>1.1272024963615108</v>
+      </c>
+      <c r="T26">
+        <v>70</v>
+      </c>
+      <c r="U26">
+        <f t="shared" si="4"/>
+        <v>2.2771406931596405E-2</v>
+      </c>
+      <c r="V26">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W26">
         <f t="shared" si="6"/>
-        <v>50</v>
-      </c>
-      <c r="M26">
-        <f t="shared" si="2"/>
-        <v>3.0066850000000005</v>
-      </c>
-      <c r="N26">
-        <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y26" t="s">
+        <v>145.45236177557203</v>
+      </c>
+      <c r="AB26" t="s">
         <v>81</v>
-      </c>
-      <c r="Z26">
-        <v>2.5</v>
-      </c>
-      <c r="AA26">
-        <v>2.5</v>
-      </c>
-      <c r="AB26">
-        <v>2.5</v>
       </c>
       <c r="AC26">
         <v>2.5</v>
@@ -1939,8 +2332,17 @@
       <c r="AE26">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF26">
+        <v>2.5</v>
+      </c>
+      <c r="AG26">
+        <v>2.5</v>
+      </c>
+      <c r="AH26">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>5</v>
       </c>
@@ -1959,41 +2361,54 @@
       <c r="G27">
         <v>0</v>
       </c>
-      <c r="I27">
-        <f>$AD$17</f>
+      <c r="J27">
+        <f>$AG$17</f>
         <v>2.9</v>
       </c>
-      <c r="J27">
-        <f>$AD$45</f>
+      <c r="L27">
+        <f>$AG$45</f>
         <v>0.75</v>
       </c>
-      <c r="K27">
+      <c r="M27">
         <f t="shared" si="0"/>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L27">
-        <f>$AD72</f>
+      <c r="O27">
+        <f>$AG72</f>
         <v>56</v>
       </c>
-      <c r="M27">
+      <c r="P27">
+        <f t="shared" si="7"/>
+        <v>1.3198285488795851</v>
+      </c>
+      <c r="Q27">
         <f t="shared" si="2"/>
-        <v>3.6104765200000011</v>
-      </c>
-      <c r="N27">
+        <v>0.9999999504359468</v>
+      </c>
+      <c r="R27">
+        <v>1</v>
+      </c>
+      <c r="S27">
         <f t="shared" si="3"/>
-        <v>0.9999999504359468</v>
-      </c>
-      <c r="Y27" t="s">
+        <v>1.3198284834635328</v>
+      </c>
+      <c r="T27">
+        <v>50</v>
+      </c>
+      <c r="U27">
+        <f t="shared" si="4"/>
+        <v>2.6392775489114419E-2</v>
+      </c>
+      <c r="V27">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W27">
+        <f t="shared" si="6"/>
+        <v>120.41703816908453</v>
+      </c>
+      <c r="AB27" t="s">
         <v>82</v>
-      </c>
-      <c r="Z27">
-        <v>0.7</v>
-      </c>
-      <c r="AA27">
-        <v>0.7</v>
-      </c>
-      <c r="AB27">
-        <v>0.7</v>
       </c>
       <c r="AC27">
         <v>0.7</v>
@@ -2004,8 +2419,17 @@
       <c r="AE27">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF27">
+        <v>0.7</v>
+      </c>
+      <c r="AG27">
+        <v>0.7</v>
+      </c>
+      <c r="AH27">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D28" t="s">
         <v>81</v>
       </c>
@@ -2018,41 +2442,54 @@
       <c r="G28">
         <v>0</v>
       </c>
-      <c r="I28">
-        <f>$AD$18</f>
+      <c r="J28">
+        <f>$AG$18</f>
         <v>2.5</v>
       </c>
-      <c r="J28">
-        <f>$AD$46</f>
+      <c r="L28">
+        <f>$AG$46</f>
         <v>0.61</v>
       </c>
-      <c r="K28">
+      <c r="M28">
         <f t="shared" si="0"/>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L28">
-        <f t="shared" ref="L28:L30" si="7">$AD73</f>
+      <c r="O28">
+        <f t="shared" ref="O28:O30" si="13">$AG73</f>
         <v>51</v>
       </c>
-      <c r="M28">
+      <c r="P28">
+        <f t="shared" si="7"/>
+        <v>0.97873546256970145</v>
+      </c>
+      <c r="Q28">
         <f t="shared" si="2"/>
-        <v>2.6155189349999994</v>
-      </c>
-      <c r="N28">
+        <v>0.99999627334682795</v>
+      </c>
+      <c r="R28">
+        <v>1</v>
+      </c>
+      <c r="S28">
         <f t="shared" si="3"/>
-        <v>0.99999627334682795</v>
-      </c>
-      <c r="Y28" t="s">
+        <v>0.97873181516208529</v>
+      </c>
+      <c r="T28">
+        <v>55</v>
+      </c>
+      <c r="U28">
+        <f t="shared" si="4"/>
+        <v>1.9980158125047207E-2</v>
+      </c>
+      <c r="V28">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W28">
+        <f t="shared" si="6"/>
+        <v>100.27541859008066</v>
+      </c>
+      <c r="AB28" t="s">
         <v>83</v>
-      </c>
-      <c r="Z28">
-        <v>0.9</v>
-      </c>
-      <c r="AA28">
-        <v>0.9</v>
-      </c>
-      <c r="AB28">
-        <v>0.9</v>
       </c>
       <c r="AC28">
         <v>0.9</v>
@@ -2063,8 +2500,17 @@
       <c r="AE28">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF28">
+        <v>0.9</v>
+      </c>
+      <c r="AG28">
+        <v>0.9</v>
+      </c>
+      <c r="AH28">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D29" t="s">
         <v>82</v>
       </c>
@@ -2077,44 +2523,57 @@
       <c r="G29">
         <v>0</v>
       </c>
-      <c r="I29">
-        <f>$AD$19</f>
+      <c r="J29">
+        <f>$AG$19</f>
         <v>1.6</v>
       </c>
-      <c r="J29">
-        <f>$AD$47</f>
+      <c r="L29">
+        <f>$AG$47</f>
         <v>0.64</v>
       </c>
-      <c r="K29">
+      <c r="M29">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L29">
+      <c r="O29">
+        <f t="shared" si="13"/>
+        <v>50</v>
+      </c>
+      <c r="P29">
         <f t="shared" si="7"/>
-        <v>50</v>
-      </c>
-      <c r="M29">
+        <v>1.0054871153505722</v>
+      </c>
+      <c r="Q29">
         <f t="shared" si="2"/>
-        <v>2.6737390000000008</v>
-      </c>
-      <c r="N29">
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R29">
+        <v>1</v>
+      </c>
+      <c r="S29">
         <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-      <c r="X29" t="s">
+        <v>0.99947830132860371</v>
+      </c>
+      <c r="T29">
+        <v>45</v>
+      </c>
+      <c r="U29">
+        <f t="shared" si="4"/>
+        <v>2.0370192064977751E-2</v>
+      </c>
+      <c r="V29">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W29">
+        <f t="shared" si="6"/>
+        <v>83.645101166814896</v>
+      </c>
+      <c r="AA29" t="s">
         <v>88</v>
       </c>
-      <c r="Y29" t="s">
+      <c r="AB29" t="s">
         <v>80</v>
-      </c>
-      <c r="Z29">
-        <v>2.5</v>
-      </c>
-      <c r="AA29">
-        <v>2.5</v>
-      </c>
-      <c r="AB29">
-        <v>2.5</v>
       </c>
       <c r="AC29">
         <v>2.5</v>
@@ -2125,8 +2584,17 @@
       <c r="AE29">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF29">
+        <v>2.5</v>
+      </c>
+      <c r="AG29">
+        <v>2.5</v>
+      </c>
+      <c r="AH29">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D30" t="s">
         <v>83</v>
       </c>
@@ -2139,41 +2607,54 @@
       <c r="G30">
         <v>0</v>
       </c>
-      <c r="I30">
-        <f>$AD$20</f>
+      <c r="J30">
+        <f>$AG$20</f>
         <v>1.7</v>
       </c>
-      <c r="J30">
-        <f>$AD$48</f>
+      <c r="L30">
+        <f>$AG$48</f>
         <v>0.72</v>
       </c>
-      <c r="K30">
+      <c r="M30">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L30">
+      <c r="O30">
+        <f t="shared" si="13"/>
+        <v>51</v>
+      </c>
+      <c r="P30">
         <f t="shared" si="7"/>
-        <v>51</v>
-      </c>
-      <c r="M30">
+        <v>1.1534721617679149</v>
+      </c>
+      <c r="Q30">
         <f t="shared" si="2"/>
-        <v>3.0824757000000003</v>
-      </c>
-      <c r="N30">
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R30">
+        <v>1</v>
+      </c>
+      <c r="S30">
         <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y30" t="s">
+        <v>1.1499094145288902</v>
+      </c>
+      <c r="T30">
+        <v>40</v>
+      </c>
+      <c r="U30">
+        <f t="shared" si="4"/>
+        <v>2.3198296993143137E-2</v>
+      </c>
+      <c r="V30">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W30">
+        <f t="shared" si="6"/>
+        <v>84.673784024972448</v>
+      </c>
+      <c r="AB30" t="s">
         <v>81</v>
-      </c>
-      <c r="Z30">
-        <v>2.5</v>
-      </c>
-      <c r="AA30">
-        <v>2.5</v>
-      </c>
-      <c r="AB30">
-        <v>2.5</v>
       </c>
       <c r="AC30">
         <v>2.5</v>
@@ -2184,8 +2665,17 @@
       <c r="AE30">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="31" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF30">
+        <v>2.5</v>
+      </c>
+      <c r="AG30">
+        <v>2.5</v>
+      </c>
+      <c r="AH30">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>6</v>
       </c>
@@ -2204,41 +2694,54 @@
       <c r="G31">
         <v>0</v>
       </c>
-      <c r="I31">
-        <f>$AE$17</f>
+      <c r="J31">
+        <f>$AH$17</f>
         <v>2.9</v>
       </c>
-      <c r="J31">
-        <f>$AE$45</f>
+      <c r="L31">
+        <f>$AH$45</f>
         <v>0.75</v>
       </c>
-      <c r="K31">
+      <c r="M31">
         <f t="shared" si="0"/>
         <v>0.5948500000000001</v>
       </c>
-      <c r="L31">
-        <f>$AE72</f>
+      <c r="O31">
+        <f>$AH72</f>
         <v>20</v>
       </c>
-      <c r="M31">
+      <c r="P31">
+        <f t="shared" si="7"/>
+        <v>0.5052226861752882</v>
+      </c>
+      <c r="Q31">
         <f t="shared" si="2"/>
-        <v>1.0684159000000002</v>
-      </c>
-      <c r="N31">
+        <v>0.9999999504359468</v>
+      </c>
+      <c r="R31">
+        <v>1</v>
+      </c>
+      <c r="S31">
         <f t="shared" si="3"/>
-        <v>0.9999999504359468</v>
-      </c>
-      <c r="Y31" t="s">
+        <v>0.50522266113440406</v>
+      </c>
+      <c r="T31">
+        <v>30</v>
+      </c>
+      <c r="U31">
+        <f t="shared" si="4"/>
+        <v>1.1078186029326796E-2</v>
+      </c>
+      <c r="V31">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W31">
+        <f t="shared" si="6"/>
+        <v>30.326534255282102</v>
+      </c>
+      <c r="AB31" t="s">
         <v>82</v>
-      </c>
-      <c r="Z31">
-        <v>1.3</v>
-      </c>
-      <c r="AA31">
-        <v>1.3</v>
-      </c>
-      <c r="AB31">
-        <v>1.3</v>
       </c>
       <c r="AC31">
         <v>1.3</v>
@@ -2249,8 +2752,17 @@
       <c r="AE31">
         <v>1.3</v>
       </c>
-    </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="AF31">
+        <v>1.3</v>
+      </c>
+      <c r="AG31">
+        <v>1.3</v>
+      </c>
+      <c r="AH31">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:34" x14ac:dyDescent="0.2">
       <c r="D32" t="s">
         <v>81</v>
       </c>
@@ -2263,41 +2775,54 @@
       <c r="G32">
         <v>0</v>
       </c>
-      <c r="I32">
-        <f>$AE$18</f>
+      <c r="J32">
+        <f>$AH$18</f>
         <v>2.5</v>
       </c>
-      <c r="J32">
-        <f>$AE$46</f>
+      <c r="L32">
+        <f>$AH$46</f>
         <v>0.61</v>
       </c>
-      <c r="K32">
+      <c r="M32">
         <f t="shared" si="0"/>
         <v>0.48354999999999998</v>
       </c>
-      <c r="L32">
-        <f t="shared" ref="L32:L34" si="8">$AE73</f>
+      <c r="O32">
+        <f t="shared" ref="O32:O34" si="14">$AH73</f>
         <v>27</v>
       </c>
-      <c r="M32">
+      <c r="P32">
+        <f t="shared" si="7"/>
+        <v>0.52017847077168489</v>
+      </c>
+      <c r="Q32">
         <f t="shared" si="2"/>
-        <v>1.185750495</v>
-      </c>
-      <c r="N32">
+        <v>0.99999627334682795</v>
+      </c>
+      <c r="R32">
+        <v>1</v>
+      </c>
+      <c r="S32">
         <f t="shared" si="3"/>
-        <v>0.99999627334682795</v>
-      </c>
-      <c r="Y32" t="s">
+        <v>0.52017653224693672</v>
+      </c>
+      <c r="T32">
+        <v>90</v>
+      </c>
+      <c r="U32">
+        <f t="shared" si="4"/>
+        <v>1.135931880624241E-2</v>
+      </c>
+      <c r="V32">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W32">
+        <f t="shared" si="6"/>
+        <v>93.288405696265798</v>
+      </c>
+      <c r="AB32" t="s">
         <v>83</v>
-      </c>
-      <c r="Z32">
-        <v>0.8</v>
-      </c>
-      <c r="AA32">
-        <v>0.8</v>
-      </c>
-      <c r="AB32">
-        <v>0.8</v>
       </c>
       <c r="AC32">
         <v>0.8</v>
@@ -2308,8 +2833,17 @@
       <c r="AE32">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="33" spans="4:31" x14ac:dyDescent="0.2">
+      <c r="AF32">
+        <v>0.8</v>
+      </c>
+      <c r="AG32">
+        <v>0.8</v>
+      </c>
+      <c r="AH32">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="33" spans="4:34" x14ac:dyDescent="0.2">
       <c r="D33" t="s">
         <v>82</v>
       </c>
@@ -2322,44 +2856,57 @@
       <c r="G33">
         <v>0</v>
       </c>
-      <c r="I33">
-        <f>$AE$19</f>
+      <c r="J33">
+        <f>$AH$19</f>
         <v>1.6</v>
       </c>
-      <c r="J33">
-        <f>$AE$47</f>
+      <c r="L33">
+        <f>$AH$47</f>
         <v>0.64</v>
       </c>
-      <c r="K33">
+      <c r="M33">
         <f t="shared" si="0"/>
         <v>0.50740000000000007</v>
       </c>
-      <c r="L33">
-        <f t="shared" si="8"/>
+      <c r="O33">
+        <f t="shared" si="14"/>
         <v>32</v>
       </c>
-      <c r="M33">
+      <c r="P33">
+        <f t="shared" si="7"/>
+        <v>0.64511931548462409</v>
+      </c>
+      <c r="Q33">
         <f t="shared" si="2"/>
-        <v>1.5343609600000003</v>
-      </c>
-      <c r="N33">
+        <v>0.99402397710499402</v>
+      </c>
+      <c r="R33">
+        <v>1</v>
+      </c>
+      <c r="S33">
         <f t="shared" si="3"/>
-        <v>0.99402397710499402</v>
-      </c>
-      <c r="X33" t="s">
+        <v>0.64126406768527744</v>
+      </c>
+      <c r="T33">
+        <v>80</v>
+      </c>
+      <c r="U33">
+        <f t="shared" si="4"/>
+        <v>1.3635764472483216E-2</v>
+      </c>
+      <c r="V33">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W33">
+        <f t="shared" si="6"/>
+        <v>99.54108064912748</v>
+      </c>
+      <c r="AA33" t="s">
         <v>89</v>
       </c>
-      <c r="Y33" t="s">
+      <c r="AB33" t="s">
         <v>80</v>
-      </c>
-      <c r="Z33">
-        <v>3.2</v>
-      </c>
-      <c r="AA33">
-        <v>3.2</v>
-      </c>
-      <c r="AB33">
-        <v>3.2</v>
       </c>
       <c r="AC33">
         <v>3.2</v>
@@ -2370,8 +2917,17 @@
       <c r="AE33">
         <v>3.2</v>
       </c>
-    </row>
-    <row r="34" spans="4:31" x14ac:dyDescent="0.2">
+      <c r="AF33">
+        <v>3.2</v>
+      </c>
+      <c r="AG33">
+        <v>3.2</v>
+      </c>
+      <c r="AH33">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="34" spans="4:34" x14ac:dyDescent="0.2">
       <c r="D34" t="s">
         <v>83</v>
       </c>
@@ -2384,41 +2940,54 @@
       <c r="G34">
         <v>0</v>
       </c>
-      <c r="I34">
-        <f>$AE$20</f>
+      <c r="J34">
+        <f>$AH$20</f>
         <v>1.7</v>
       </c>
-      <c r="J34">
-        <f>$AE$48</f>
+      <c r="L34">
+        <f>$AH$48</f>
         <v>0.72</v>
       </c>
-      <c r="K34">
+      <c r="M34">
         <f t="shared" si="0"/>
         <v>0.57100000000000006</v>
       </c>
-      <c r="L34">
-        <f t="shared" si="8"/>
+      <c r="O34">
+        <f t="shared" si="14"/>
         <v>34</v>
       </c>
-      <c r="M34">
-        <f>(104.7 * K34 + 0.307 * L34- 15) * L34 * 10^-3</f>
-        <v>1.8775378000000005</v>
-      </c>
-      <c r="N34">
+      <c r="P34">
+        <f t="shared" si="7"/>
+        <v>0.77753323213623582</v>
+      </c>
+      <c r="Q34">
+        <f t="shared" si="2"/>
+        <v>0.99691128459176326</v>
+      </c>
+      <c r="R34">
+        <v>1</v>
+      </c>
+      <c r="S34">
         <f t="shared" si="3"/>
-        <v>0.99691128459176326</v>
-      </c>
-      <c r="Y34" t="s">
+        <v>0.77513165326172051</v>
+      </c>
+      <c r="T34">
+        <v>70</v>
+      </c>
+      <c r="U34">
+        <f t="shared" si="4"/>
+        <v>1.6152475081320346E-2</v>
+      </c>
+      <c r="V34">
+        <f t="shared" si="5"/>
+        <v>91.25</v>
+      </c>
+      <c r="W34">
+        <f t="shared" si="6"/>
+        <v>103.17393458193371</v>
+      </c>
+      <c r="AB34" t="s">
         <v>81</v>
-      </c>
-      <c r="Z34">
-        <v>3</v>
-      </c>
-      <c r="AA34">
-        <v>3</v>
-      </c>
-      <c r="AB34">
-        <v>3</v>
       </c>
       <c r="AC34">
         <v>3</v>
@@ -2429,19 +2998,19 @@
       <c r="AE34">
         <v>3</v>
       </c>
-    </row>
-    <row r="35" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y35" t="s">
+      <c r="AF34">
+        <v>3</v>
+      </c>
+      <c r="AG34">
+        <v>3</v>
+      </c>
+      <c r="AH34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB35" t="s">
         <v>82</v>
-      </c>
-      <c r="Z35">
-        <v>1.8</v>
-      </c>
-      <c r="AA35">
-        <v>1.8</v>
-      </c>
-      <c r="AB35">
-        <v>1.8</v>
       </c>
       <c r="AC35">
         <v>1.8</v>
@@ -2452,19 +3021,19 @@
       <c r="AE35">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="36" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y36" t="s">
+      <c r="AF35">
+        <v>1.8</v>
+      </c>
+      <c r="AG35">
+        <v>1.8</v>
+      </c>
+      <c r="AH35">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="36" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB36" t="s">
         <v>83</v>
-      </c>
-      <c r="Z36">
-        <v>1</v>
-      </c>
-      <c r="AA36">
-        <v>1</v>
-      </c>
-      <c r="AB36">
-        <v>1</v>
       </c>
       <c r="AC36">
         <v>1</v>
@@ -2475,22 +3044,22 @@
       <c r="AE36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="X37" t="s">
+      <c r="AF36">
+        <v>1</v>
+      </c>
+      <c r="AG36">
+        <v>1</v>
+      </c>
+      <c r="AH36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AA37" t="s">
         <v>90</v>
       </c>
-      <c r="Y37" t="s">
+      <c r="AB37" t="s">
         <v>80</v>
-      </c>
-      <c r="Z37">
-        <v>3.5</v>
-      </c>
-      <c r="AA37">
-        <v>3.5</v>
-      </c>
-      <c r="AB37">
-        <v>3.5</v>
       </c>
       <c r="AC37">
         <v>3.5</v>
@@ -2501,19 +3070,19 @@
       <c r="AE37">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="38" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y38" t="s">
+      <c r="AF37">
+        <v>3.5</v>
+      </c>
+      <c r="AG37">
+        <v>3.5</v>
+      </c>
+      <c r="AH37">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="38" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB38" t="s">
         <v>81</v>
-      </c>
-      <c r="Z38">
-        <v>1.5</v>
-      </c>
-      <c r="AA38">
-        <v>1.5</v>
-      </c>
-      <c r="AB38">
-        <v>1.5</v>
       </c>
       <c r="AC38">
         <v>1.5</v>
@@ -2524,19 +3093,19 @@
       <c r="AE38">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="39" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y39" t="s">
+      <c r="AF38">
+        <v>1.5</v>
+      </c>
+      <c r="AG38">
+        <v>1.5</v>
+      </c>
+      <c r="AH38">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="39" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB39" t="s">
         <v>82</v>
-      </c>
-      <c r="Z39">
-        <v>0.7</v>
-      </c>
-      <c r="AA39">
-        <v>0.7</v>
-      </c>
-      <c r="AB39">
-        <v>0.7</v>
       </c>
       <c r="AC39">
         <v>0.7</v>
@@ -2547,19 +3116,19 @@
       <c r="AE39">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="40" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y40" t="s">
+      <c r="AF39">
+        <v>0.7</v>
+      </c>
+      <c r="AG39">
+        <v>0.7</v>
+      </c>
+      <c r="AH39">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="40" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB40" t="s">
         <v>83</v>
-      </c>
-      <c r="Z40">
-        <v>1.2</v>
-      </c>
-      <c r="AA40">
-        <v>1.2</v>
-      </c>
-      <c r="AB40">
-        <v>1.2</v>
       </c>
       <c r="AC40">
         <v>1.2</v>
@@ -2570,29 +3139,29 @@
       <c r="AE40">
         <v>1.2</v>
       </c>
-    </row>
-    <row r="43" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y43" t="s">
+      <c r="AF40">
+        <v>1.2</v>
+      </c>
+      <c r="AG40">
+        <v>1.2</v>
+      </c>
+      <c r="AH40">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="43" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB43" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y44" t="s">
+    <row r="44" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB44" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y45" t="s">
+    <row r="45" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB45" t="s">
         <v>80</v>
-      </c>
-      <c r="Z45">
-        <v>0.75</v>
-      </c>
-      <c r="AA45">
-        <v>0.75</v>
-      </c>
-      <c r="AB45">
-        <v>0.75</v>
       </c>
       <c r="AC45">
         <v>0.75</v>
@@ -2603,19 +3172,19 @@
       <c r="AE45">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="46" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y46" t="s">
+      <c r="AF45">
+        <v>0.75</v>
+      </c>
+      <c r="AG45">
+        <v>0.75</v>
+      </c>
+      <c r="AH45">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="46" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB46" t="s">
         <v>81</v>
-      </c>
-      <c r="Z46">
-        <v>0.61</v>
-      </c>
-      <c r="AA46">
-        <v>0.61</v>
-      </c>
-      <c r="AB46">
-        <v>0.61</v>
       </c>
       <c r="AC46">
         <v>0.61</v>
@@ -2626,19 +3195,19 @@
       <c r="AE46">
         <v>0.61</v>
       </c>
-    </row>
-    <row r="47" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y47" t="s">
+      <c r="AF46">
+        <v>0.61</v>
+      </c>
+      <c r="AG46">
+        <v>0.61</v>
+      </c>
+      <c r="AH46">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="47" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB47" t="s">
         <v>82</v>
-      </c>
-      <c r="Z47">
-        <v>0.64</v>
-      </c>
-      <c r="AA47">
-        <v>0.64</v>
-      </c>
-      <c r="AB47">
-        <v>0.64</v>
       </c>
       <c r="AC47">
         <v>0.64</v>
@@ -2649,19 +3218,19 @@
       <c r="AE47">
         <v>0.64</v>
       </c>
-    </row>
-    <row r="48" spans="4:31" x14ac:dyDescent="0.2">
-      <c r="Y48" t="s">
+      <c r="AF47">
+        <v>0.64</v>
+      </c>
+      <c r="AG47">
+        <v>0.64</v>
+      </c>
+      <c r="AH47">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="48" spans="4:34" x14ac:dyDescent="0.2">
+      <c r="AB48" t="s">
         <v>83</v>
-      </c>
-      <c r="Z48">
-        <v>0.72</v>
-      </c>
-      <c r="AA48">
-        <v>0.72</v>
-      </c>
-      <c r="AB48">
-        <v>0.72</v>
       </c>
       <c r="AC48">
         <v>0.72</v>
@@ -2672,19 +3241,19 @@
       <c r="AE48">
         <v>0.72</v>
       </c>
-    </row>
-    <row r="49" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y49" t="s">
+      <c r="AF48">
+        <v>0.72</v>
+      </c>
+      <c r="AG48">
+        <v>0.72</v>
+      </c>
+      <c r="AH48">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="49" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB49" t="s">
         <v>80</v>
-      </c>
-      <c r="Z49">
-        <v>0.51</v>
-      </c>
-      <c r="AA49">
-        <v>0.51</v>
-      </c>
-      <c r="AB49">
-        <v>0.51</v>
       </c>
       <c r="AC49">
         <v>0.51</v>
@@ -2695,19 +3264,19 @@
       <c r="AE49">
         <v>0.51</v>
       </c>
-    </row>
-    <row r="50" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y50" t="s">
+      <c r="AF49">
+        <v>0.51</v>
+      </c>
+      <c r="AG49">
+        <v>0.51</v>
+      </c>
+      <c r="AH49">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="50" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB50" t="s">
         <v>81</v>
-      </c>
-      <c r="Z50">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA50">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB50">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC50">
         <v>0.55000000000000004</v>
@@ -2718,19 +3287,19 @@
       <c r="AE50">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="51" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y51" t="s">
+      <c r="AF50">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG50">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH50">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="51" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB51" t="s">
         <v>82</v>
-      </c>
-      <c r="Z51">
-        <v>0.59</v>
-      </c>
-      <c r="AA51">
-        <v>0.59</v>
-      </c>
-      <c r="AB51">
-        <v>0.59</v>
       </c>
       <c r="AC51">
         <v>0.59</v>
@@ -2741,19 +3310,19 @@
       <c r="AE51">
         <v>0.59</v>
       </c>
-    </row>
-    <row r="52" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y52" t="s">
+      <c r="AF51">
+        <v>0.59</v>
+      </c>
+      <c r="AG51">
+        <v>0.59</v>
+      </c>
+      <c r="AH51">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="52" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB52" t="s">
         <v>83</v>
-      </c>
-      <c r="Z52">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="AA52">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="AB52">
-        <v>0.57999999999999996</v>
       </c>
       <c r="AC52">
         <v>0.57999999999999996</v>
@@ -2764,19 +3333,19 @@
       <c r="AE52">
         <v>0.57999999999999996</v>
       </c>
-    </row>
-    <row r="53" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y53" t="s">
+      <c r="AF52">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="AG52">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="AH52">
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB53" t="s">
         <v>80</v>
-      </c>
-      <c r="Z53">
-        <v>0.7</v>
-      </c>
-      <c r="AA53">
-        <v>0.7</v>
-      </c>
-      <c r="AB53">
-        <v>0.7</v>
       </c>
       <c r="AC53">
         <v>0.7</v>
@@ -2787,19 +3356,19 @@
       <c r="AE53">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="54" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y54" t="s">
+      <c r="AF53">
+        <v>0.7</v>
+      </c>
+      <c r="AG53">
+        <v>0.7</v>
+      </c>
+      <c r="AH53">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="54" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB54" t="s">
         <v>81</v>
-      </c>
-      <c r="Z54">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA54">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB54">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC54">
         <v>0.55000000000000004</v>
@@ -2810,19 +3379,19 @@
       <c r="AE54">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="55" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y55" t="s">
+      <c r="AF54">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG54">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH54">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="55" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB55" t="s">
         <v>82</v>
-      </c>
-      <c r="Z55">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA55">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB55">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC55">
         <v>0.55000000000000004</v>
@@ -2833,19 +3402,19 @@
       <c r="AE55">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="56" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y56" t="s">
+      <c r="AF55">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG55">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH55">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="56" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB56" t="s">
         <v>83</v>
-      </c>
-      <c r="Z56">
-        <v>0.75</v>
-      </c>
-      <c r="AA56">
-        <v>0.75</v>
-      </c>
-      <c r="AB56">
-        <v>0.75</v>
       </c>
       <c r="AC56">
         <v>0.75</v>
@@ -2856,19 +3425,19 @@
       <c r="AE56">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="57" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y57" t="s">
+      <c r="AF56">
+        <v>0.75</v>
+      </c>
+      <c r="AG56">
+        <v>0.75</v>
+      </c>
+      <c r="AH56">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="57" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB57" t="s">
         <v>80</v>
-      </c>
-      <c r="Z57">
-        <v>0.75</v>
-      </c>
-      <c r="AA57">
-        <v>0.75</v>
-      </c>
-      <c r="AB57">
-        <v>0.75</v>
       </c>
       <c r="AC57">
         <v>0.75</v>
@@ -2879,19 +3448,19 @@
       <c r="AE57">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="58" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y58" t="s">
+      <c r="AF57">
+        <v>0.75</v>
+      </c>
+      <c r="AG57">
+        <v>0.75</v>
+      </c>
+      <c r="AH57">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="58" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB58" t="s">
         <v>81</v>
-      </c>
-      <c r="Z58">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA58">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB58">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC58">
         <v>0.55000000000000004</v>
@@ -2902,19 +3471,19 @@
       <c r="AE58">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="59" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y59" t="s">
+      <c r="AF58">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG58">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH58">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="59" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB59" t="s">
         <v>82</v>
-      </c>
-      <c r="Z59">
-        <v>0.67</v>
-      </c>
-      <c r="AA59">
-        <v>0.67</v>
-      </c>
-      <c r="AB59">
-        <v>0.67</v>
       </c>
       <c r="AC59">
         <v>0.67</v>
@@ -2925,19 +3494,19 @@
       <c r="AE59">
         <v>0.67</v>
       </c>
-    </row>
-    <row r="60" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y60" t="s">
+      <c r="AF59">
+        <v>0.67</v>
+      </c>
+      <c r="AG59">
+        <v>0.67</v>
+      </c>
+      <c r="AH59">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="60" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB60" t="s">
         <v>83</v>
-      </c>
-      <c r="Z60">
-        <v>0.7</v>
-      </c>
-      <c r="AA60">
-        <v>0.7</v>
-      </c>
-      <c r="AB60">
-        <v>0.7</v>
       </c>
       <c r="AC60">
         <v>0.7</v>
@@ -2948,19 +3517,19 @@
       <c r="AE60">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="61" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y61" t="s">
+      <c r="AF60">
+        <v>0.7</v>
+      </c>
+      <c r="AG60">
+        <v>0.7</v>
+      </c>
+      <c r="AH60">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="61" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB61" t="s">
         <v>80</v>
-      </c>
-      <c r="Z61">
-        <v>0.7</v>
-      </c>
-      <c r="AA61">
-        <v>0.7</v>
-      </c>
-      <c r="AB61">
-        <v>0.7</v>
       </c>
       <c r="AC61">
         <v>0.7</v>
@@ -2971,19 +3540,19 @@
       <c r="AE61">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="62" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y62" t="s">
+      <c r="AF61">
+        <v>0.7</v>
+      </c>
+      <c r="AG61">
+        <v>0.7</v>
+      </c>
+      <c r="AH61">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="62" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB62" t="s">
         <v>81</v>
-      </c>
-      <c r="Z62">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA62">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB62">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC62">
         <v>0.55000000000000004</v>
@@ -2994,19 +3563,19 @@
       <c r="AE62">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="63" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y63" t="s">
+      <c r="AF62">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG62">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH62">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="63" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB63" t="s">
         <v>82</v>
-      </c>
-      <c r="Z63">
-        <v>0.65</v>
-      </c>
-      <c r="AA63">
-        <v>0.65</v>
-      </c>
-      <c r="AB63">
-        <v>0.65</v>
       </c>
       <c r="AC63">
         <v>0.65</v>
@@ -3017,19 +3586,19 @@
       <c r="AE63">
         <v>0.65</v>
       </c>
-    </row>
-    <row r="64" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y64" t="s">
+      <c r="AF63">
+        <v>0.65</v>
+      </c>
+      <c r="AG63">
+        <v>0.65</v>
+      </c>
+      <c r="AH63">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="64" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB64" t="s">
         <v>83</v>
-      </c>
-      <c r="Z64">
-        <v>0.6</v>
-      </c>
-      <c r="AA64">
-        <v>0.6</v>
-      </c>
-      <c r="AB64">
-        <v>0.6</v>
       </c>
       <c r="AC64">
         <v>0.6</v>
@@ -3040,19 +3609,19 @@
       <c r="AE64">
         <v>0.6</v>
       </c>
-    </row>
-    <row r="65" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y65" t="s">
+      <c r="AF64">
+        <v>0.6</v>
+      </c>
+      <c r="AG64">
+        <v>0.6</v>
+      </c>
+      <c r="AH64">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="65" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB65" t="s">
         <v>80</v>
-      </c>
-      <c r="Z65">
-        <v>0.73</v>
-      </c>
-      <c r="AA65">
-        <v>0.73</v>
-      </c>
-      <c r="AB65">
-        <v>0.73</v>
       </c>
       <c r="AC65">
         <v>0.73</v>
@@ -3063,19 +3632,19 @@
       <c r="AE65">
         <v>0.73</v>
       </c>
-    </row>
-    <row r="66" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y66" t="s">
+      <c r="AF65">
+        <v>0.73</v>
+      </c>
+      <c r="AG65">
+        <v>0.73</v>
+      </c>
+      <c r="AH65">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="66" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB66" t="s">
         <v>81</v>
-      </c>
-      <c r="Z66">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AA66">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="AB66">
-        <v>0.55000000000000004</v>
       </c>
       <c r="AC66">
         <v>0.55000000000000004</v>
@@ -3086,22 +3655,22 @@
       <c r="AE66">
         <v>0.55000000000000004</v>
       </c>
-    </row>
-    <row r="67" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y67" t="s">
+      <c r="AF66">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AG66">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="AH66">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="67" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB67" t="s">
         <v>82</v>
       </c>
-      <c r="Z67">
+      <c r="AC67">
         <v>0.5</v>
-      </c>
-      <c r="AA67">
-        <v>0.5</v>
-      </c>
-      <c r="AB67">
-        <v>0.7</v>
-      </c>
-      <c r="AC67">
-        <v>0.7</v>
       </c>
       <c r="AD67">
         <v>0.5</v>
@@ -3109,19 +3678,19 @@
       <c r="AE67">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="68" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y68" t="s">
+      <c r="AF67">
+        <v>0.7</v>
+      </c>
+      <c r="AG67">
+        <v>0.5</v>
+      </c>
+      <c r="AH67">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="68" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB68" t="s">
         <v>83</v>
-      </c>
-      <c r="Z68">
-        <v>0.76</v>
-      </c>
-      <c r="AA68">
-        <v>0.76</v>
-      </c>
-      <c r="AB68">
-        <v>0.76</v>
       </c>
       <c r="AC68">
         <v>0.76</v>
@@ -3132,571 +3701,580 @@
       <c r="AE68">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="71" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y71" t="s">
+      <c r="AF68">
+        <v>0.76</v>
+      </c>
+      <c r="AG68">
+        <v>0.76</v>
+      </c>
+      <c r="AH68">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="71" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB71" t="s">
         <v>94</v>
       </c>
-      <c r="Z71" t="s">
+      <c r="AC71" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="72" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y72" t="s">
+    <row r="72" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB72" t="s">
         <v>80</v>
       </c>
-      <c r="Z72">
+      <c r="AC72">
         <v>75</v>
       </c>
-      <c r="AA72">
+      <c r="AD72">
         <v>62</v>
       </c>
-      <c r="AB72">
+      <c r="AE72">
         <v>44</v>
       </c>
-      <c r="AC72">
+      <c r="AF72">
         <v>54</v>
       </c>
-      <c r="AD72">
+      <c r="AG72">
         <v>56</v>
       </c>
-      <c r="AE72">
+      <c r="AH72">
         <v>20</v>
       </c>
     </row>
-    <row r="73" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y73" t="s">
+    <row r="73" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB73" t="s">
         <v>81</v>
       </c>
-      <c r="Z73">
+      <c r="AC73">
         <v>75</v>
       </c>
-      <c r="AA73">
+      <c r="AD73">
         <v>55</v>
       </c>
-      <c r="AB73">
+      <c r="AE73">
         <v>42</v>
       </c>
-      <c r="AC73">
+      <c r="AF73">
         <v>49</v>
       </c>
-      <c r="AD73">
+      <c r="AG73">
         <v>51</v>
       </c>
-      <c r="AE73">
+      <c r="AH73">
         <v>27</v>
       </c>
     </row>
-    <row r="74" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y74" t="s">
+    <row r="74" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB74" t="s">
         <v>82</v>
       </c>
-      <c r="Z74">
+      <c r="AC74">
         <v>69</v>
       </c>
-      <c r="AA74">
+      <c r="AD74">
         <v>55</v>
       </c>
-      <c r="AB74">
+      <c r="AE74">
         <v>43</v>
       </c>
-      <c r="AC74">
+      <c r="AF74">
         <v>50</v>
       </c>
-      <c r="AD74">
+      <c r="AG74">
         <v>50</v>
       </c>
-      <c r="AE74">
+      <c r="AH74">
         <v>32</v>
       </c>
     </row>
-    <row r="75" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y75" t="s">
+    <row r="75" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB75" t="s">
         <v>83</v>
       </c>
-      <c r="Z75">
+      <c r="AC75">
         <v>69</v>
       </c>
-      <c r="AA75">
+      <c r="AD75">
         <v>55</v>
       </c>
-      <c r="AB75">
+      <c r="AE75">
         <v>45</v>
       </c>
-      <c r="AC75">
+      <c r="AF75">
         <v>50</v>
       </c>
-      <c r="AD75">
+      <c r="AG75">
         <v>51</v>
       </c>
-      <c r="AE75">
+      <c r="AH75">
         <v>34</v>
       </c>
     </row>
-    <row r="76" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y76" t="s">
+    <row r="76" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB76" t="s">
         <v>80</v>
       </c>
-      <c r="Z76">
+      <c r="AC76">
         <v>58</v>
       </c>
-      <c r="AA76">
+      <c r="AD76">
         <v>50</v>
       </c>
-      <c r="AB76">
+      <c r="AE76">
         <v>35</v>
       </c>
-      <c r="AC76">
+      <c r="AF76">
         <v>40</v>
       </c>
-      <c r="AD76">
+      <c r="AG76">
         <v>45</v>
       </c>
-      <c r="AE76">
+      <c r="AH76">
         <v>20</v>
       </c>
     </row>
-    <row r="77" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y77" t="s">
+    <row r="77" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB77" t="s">
         <v>81</v>
       </c>
-      <c r="Z77">
+      <c r="AC77">
         <v>61</v>
       </c>
-      <c r="AA77">
+      <c r="AD77">
         <v>55</v>
       </c>
-      <c r="AB77">
+      <c r="AE77">
         <v>40</v>
       </c>
-      <c r="AC77">
+      <c r="AF77">
         <v>45</v>
       </c>
-      <c r="AD77">
+      <c r="AG77">
         <v>50</v>
       </c>
-      <c r="AE77">
+      <c r="AH77">
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y78" t="s">
+    <row r="78" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB78" t="s">
         <v>82</v>
       </c>
-      <c r="Z78">
+      <c r="AC78">
         <v>63</v>
       </c>
-      <c r="AA78">
+      <c r="AD78">
         <v>55</v>
       </c>
-      <c r="AB78">
+      <c r="AE78">
         <v>40</v>
       </c>
-      <c r="AC78">
+      <c r="AF78">
         <v>45</v>
       </c>
-      <c r="AD78">
+      <c r="AG78">
         <v>50</v>
       </c>
-      <c r="AE78">
+      <c r="AH78">
         <v>20</v>
       </c>
     </row>
-    <row r="79" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y79" t="s">
+    <row r="79" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB79" t="s">
         <v>83</v>
       </c>
-      <c r="Z79">
+      <c r="AC79">
         <v>60</v>
       </c>
-      <c r="AA79">
+      <c r="AD79">
         <v>50</v>
       </c>
-      <c r="AB79">
+      <c r="AE79">
         <v>35</v>
       </c>
-      <c r="AC79">
+      <c r="AF79">
         <v>42</v>
       </c>
-      <c r="AD79">
+      <c r="AG79">
         <v>48</v>
       </c>
-      <c r="AE79">
+      <c r="AH79">
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y80" t="s">
+    <row r="80" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB80" t="s">
         <v>80</v>
       </c>
-      <c r="Z80">
+      <c r="AC80">
         <v>80</v>
       </c>
-      <c r="AA80">
+      <c r="AD80">
         <v>70</v>
       </c>
-      <c r="AB80">
+      <c r="AE80">
         <v>52</v>
       </c>
-      <c r="AC80">
+      <c r="AF80">
         <v>55</v>
       </c>
-      <c r="AD80">
+      <c r="AG80">
         <v>55</v>
       </c>
-      <c r="AE80">
+      <c r="AH80">
         <v>40</v>
       </c>
     </row>
-    <row r="81" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y81" t="s">
+    <row r="81" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB81" t="s">
         <v>81</v>
       </c>
-      <c r="Z81">
+      <c r="AC81">
         <v>70</v>
       </c>
-      <c r="AA81">
+      <c r="AD81">
         <v>65</v>
       </c>
-      <c r="AB81">
+      <c r="AE81">
         <v>52</v>
       </c>
-      <c r="AC81">
+      <c r="AF81">
         <v>55</v>
       </c>
-      <c r="AD81">
+      <c r="AG81">
         <v>55</v>
       </c>
-      <c r="AE81">
+      <c r="AH81">
         <v>45</v>
       </c>
     </row>
-    <row r="82" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y82" t="s">
+    <row r="82" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB82" t="s">
         <v>82</v>
       </c>
-      <c r="Z82">
+      <c r="AC82">
         <v>70</v>
       </c>
-      <c r="AA82">
+      <c r="AD82">
         <v>60</v>
       </c>
-      <c r="AB82">
+      <c r="AE82">
         <v>52</v>
       </c>
-      <c r="AC82">
+      <c r="AF82">
         <v>55</v>
       </c>
-      <c r="AD82">
+      <c r="AG82">
         <v>55</v>
       </c>
-      <c r="AE82">
+      <c r="AH82">
         <v>20</v>
       </c>
     </row>
-    <row r="83" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y83" t="s">
+    <row r="83" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB83" t="s">
         <v>83</v>
       </c>
-      <c r="Z83">
+      <c r="AC83">
         <v>70</v>
       </c>
-      <c r="AA83">
+      <c r="AD83">
         <v>60</v>
       </c>
-      <c r="AB83">
+      <c r="AE83">
         <v>52</v>
       </c>
-      <c r="AC83">
+      <c r="AF83">
         <v>55</v>
       </c>
-      <c r="AD83">
+      <c r="AG83">
         <v>55</v>
       </c>
-      <c r="AE83">
+      <c r="AH83">
         <v>30</v>
       </c>
     </row>
-    <row r="84" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y84" t="s">
+    <row r="84" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB84" t="s">
         <v>80</v>
       </c>
-      <c r="Z84">
+      <c r="AC84">
         <v>90</v>
       </c>
-      <c r="AA84">
+      <c r="AD84">
         <v>55</v>
       </c>
-      <c r="AB84">
+      <c r="AE84">
         <v>45</v>
       </c>
-      <c r="AC84">
+      <c r="AF84">
         <v>50</v>
       </c>
-      <c r="AD84">
+      <c r="AG84">
         <v>50</v>
       </c>
-      <c r="AE84">
+      <c r="AH84">
         <v>14</v>
       </c>
     </row>
-    <row r="85" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y85" t="s">
+    <row r="85" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB85" t="s">
         <v>81</v>
       </c>
-      <c r="Z85">
+      <c r="AC85">
         <v>90</v>
       </c>
-      <c r="AA85">
+      <c r="AD85">
         <v>55</v>
       </c>
-      <c r="AB85">
+      <c r="AE85">
         <v>45</v>
       </c>
-      <c r="AC85">
+      <c r="AF85">
         <v>50</v>
       </c>
-      <c r="AD85">
+      <c r="AG85">
         <v>50</v>
       </c>
-      <c r="AE85">
+      <c r="AH85">
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y86" t="s">
+    <row r="86" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB86" t="s">
         <v>82</v>
       </c>
-      <c r="Z86">
+      <c r="AC86">
         <v>75</v>
-      </c>
-      <c r="AA86">
-        <v>50</v>
-      </c>
-      <c r="AB86">
-        <v>45</v>
-      </c>
-      <c r="AC86">
-        <v>50</v>
       </c>
       <c r="AD86">
         <v>50</v>
       </c>
       <c r="AE86">
+        <v>45</v>
+      </c>
+      <c r="AF86">
+        <v>50</v>
+      </c>
+      <c r="AG86">
+        <v>50</v>
+      </c>
+      <c r="AH86">
         <v>36</v>
       </c>
     </row>
-    <row r="87" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y87" t="s">
+    <row r="87" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB87" t="s">
         <v>83</v>
       </c>
-      <c r="Z87">
+      <c r="AC87">
         <v>75</v>
       </c>
-      <c r="AA87">
+      <c r="AD87">
         <v>45</v>
       </c>
-      <c r="AB87">
+      <c r="AE87">
         <v>50</v>
       </c>
-      <c r="AC87">
+      <c r="AF87">
         <v>55</v>
       </c>
-      <c r="AD87">
+      <c r="AG87">
         <v>50</v>
       </c>
-      <c r="AE87">
+      <c r="AH87">
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y88" t="s">
+    <row r="88" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB88" t="s">
         <v>80</v>
       </c>
-      <c r="Z88">
+      <c r="AC88">
         <v>70</v>
       </c>
-      <c r="AA88">
+      <c r="AD88">
         <v>60</v>
       </c>
-      <c r="AB88">
+      <c r="AE88">
         <v>50</v>
       </c>
-      <c r="AC88">
+      <c r="AF88">
         <v>55</v>
       </c>
-      <c r="AD88">
+      <c r="AG88">
         <v>50</v>
       </c>
-      <c r="AE88">
+      <c r="AH88">
         <v>22</v>
       </c>
     </row>
-    <row r="89" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y89" t="s">
+    <row r="89" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB89" t="s">
         <v>81</v>
       </c>
-      <c r="Z89">
+      <c r="AC89">
         <v>65</v>
       </c>
-      <c r="AA89">
+      <c r="AD89">
         <v>55</v>
       </c>
-      <c r="AB89">
+      <c r="AE89">
         <v>45</v>
       </c>
-      <c r="AC89">
+      <c r="AF89">
         <v>50</v>
       </c>
-      <c r="AD89">
+      <c r="AG89">
         <v>50</v>
       </c>
-      <c r="AE89">
+      <c r="AH89">
         <v>28</v>
       </c>
     </row>
-    <row r="90" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y90" t="s">
+    <row r="90" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB90" t="s">
         <v>82</v>
       </c>
-      <c r="Z90">
+      <c r="AC90">
         <v>65</v>
       </c>
-      <c r="AA90">
+      <c r="AD90">
         <v>52</v>
       </c>
-      <c r="AB90">
+      <c r="AE90">
         <v>43</v>
       </c>
-      <c r="AC90">
+      <c r="AF90">
         <v>48</v>
       </c>
-      <c r="AD90">
+      <c r="AG90">
         <v>50</v>
       </c>
-      <c r="AE90">
+      <c r="AH90">
         <v>33</v>
       </c>
     </row>
-    <row r="91" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y91" t="s">
+    <row r="91" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB91" t="s">
         <v>83</v>
       </c>
-      <c r="Z91">
+      <c r="AC91">
         <v>60</v>
-      </c>
-      <c r="AA91">
-        <v>50</v>
-      </c>
-      <c r="AB91">
-        <v>40</v>
-      </c>
-      <c r="AC91">
-        <v>45</v>
       </c>
       <c r="AD91">
         <v>50</v>
       </c>
       <c r="AE91">
+        <v>40</v>
+      </c>
+      <c r="AF91">
+        <v>45</v>
+      </c>
+      <c r="AG91">
+        <v>50</v>
+      </c>
+      <c r="AH91">
         <v>35</v>
       </c>
     </row>
-    <row r="92" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y92" t="s">
+    <row r="92" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB92" t="s">
         <v>80</v>
       </c>
-      <c r="Z92">
+      <c r="AC92">
         <v>75</v>
       </c>
-      <c r="AA92">
+      <c r="AD92">
         <v>60</v>
       </c>
-      <c r="AB92">
+      <c r="AE92">
         <v>50</v>
       </c>
-      <c r="AC92">
+      <c r="AF92">
         <v>55</v>
       </c>
-      <c r="AD92">
+      <c r="AG92">
         <v>55</v>
       </c>
-      <c r="AE92">
+      <c r="AH92">
         <v>30</v>
       </c>
     </row>
-    <row r="93" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y93" t="s">
+    <row r="93" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB93" t="s">
         <v>81</v>
       </c>
-      <c r="Z93">
+      <c r="AC93">
         <v>65</v>
       </c>
-      <c r="AA93">
+      <c r="AD93">
         <v>55</v>
       </c>
-      <c r="AB93">
+      <c r="AE93">
         <v>45</v>
       </c>
-      <c r="AC93">
+      <c r="AF93">
         <v>50</v>
       </c>
-      <c r="AD93">
+      <c r="AG93">
         <v>50</v>
       </c>
-      <c r="AE93">
+      <c r="AH93">
         <v>30</v>
       </c>
     </row>
-    <row r="94" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y94" t="s">
+    <row r="94" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB94" t="s">
         <v>82</v>
       </c>
-      <c r="Z94">
+      <c r="AC94">
         <v>65</v>
       </c>
-      <c r="AA94">
+      <c r="AD94">
         <v>48</v>
       </c>
-      <c r="AB94">
+      <c r="AE94">
         <v>40</v>
       </c>
-      <c r="AC94">
+      <c r="AF94">
         <v>45</v>
       </c>
-      <c r="AD94">
+      <c r="AG94">
         <v>45</v>
       </c>
-      <c r="AE94">
+      <c r="AH94">
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="25:31" x14ac:dyDescent="0.2">
-      <c r="Y95" t="s">
+    <row r="95" spans="28:34" x14ac:dyDescent="0.2">
+      <c r="AB95" t="s">
         <v>83</v>
       </c>
-      <c r="Z95">
+      <c r="AC95">
         <v>65</v>
       </c>
-      <c r="AA95">
+      <c r="AD95">
         <v>48</v>
       </c>
-      <c r="AB95">
+      <c r="AE95">
         <v>45</v>
       </c>
-      <c r="AC95">
+      <c r="AF95">
         <v>50</v>
       </c>
-      <c r="AD95">
+      <c r="AG95">
         <v>50</v>
       </c>
-      <c r="AE95">
+      <c r="AH95">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="E2:T10 H11 K11 M11 O11:T11" numberStoredAsText="1"/>
+    <ignoredError sqref="O2:W10 H11 M11 U11 L2:M10 J2:J10 E2:H10" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(calculators): test case for monthly inputs for sheep methane passing
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.4-sheep-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.4-sheep-enteric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{7C0BEE95-3EFB-8E4B-A8AD-17CF5E770664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{6AC5A6E4-D5E1-564B-8B69-5F8E1D530314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51200" yWindow="12780" windowWidth="28800" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18007,7 +18007,7 @@
       </c>
       <c r="Z331">
         <f>SUM(Y331:Y378)*10^-3</f>
-        <v>1.0980991968840577</v>
+        <v>1.0851276670917087</v>
       </c>
     </row>
     <row r="332" spans="1:26" x14ac:dyDescent="0.2">
@@ -18198,6 +18198,10 @@
         <f>U334*V334*X334</f>
         <v>17.691018797834467</v>
       </c>
+      <c r="Z334">
+        <f>SUM(Y331:Y342)</f>
+        <v>247.00396212739781</v>
+      </c>
     </row>
     <row r="335" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D335" t="s">
@@ -18328,7 +18332,7 @@
         <v>15.287592025605933</v>
       </c>
     </row>
-    <row r="337" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D337" t="s">
         <v>83</v>
       </c>
@@ -18391,7 +18395,7 @@
         <v>18.956614111751357</v>
       </c>
     </row>
-    <row r="338" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D338" t="s">
         <v>83</v>
       </c>
@@ -18454,7 +18458,7 @@
         <v>18.956614111751357</v>
       </c>
     </row>
-    <row r="339" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D339" t="s">
         <v>80</v>
       </c>
@@ -18520,7 +18524,7 @@
         <v>25.638720846356733</v>
       </c>
     </row>
-    <row r="340" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D340" t="s">
         <v>80</v>
       </c>
@@ -18583,7 +18587,7 @@
         <v>27.818012118297055</v>
       </c>
     </row>
-    <row r="341" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D341" t="s">
         <v>80</v>
       </c>
@@ -18646,7 +18650,7 @@
         <v>25.638720846356733</v>
       </c>
     </row>
-    <row r="342" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D342" t="s">
         <v>81</v>
       </c>
@@ -18709,7 +18713,7 @@
         <v>20.823468255979723</v>
       </c>
     </row>
-    <row r="343" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A343">
         <v>2</v>
       </c>
@@ -18777,8 +18781,12 @@
         <f>U343*V343*X343</f>
         <v>36.497402688737196</v>
       </c>
-    </row>
-    <row r="344" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="Z343">
+        <f>SUM(Y343:Y354)</f>
+        <v>398.56804122405254</v>
+      </c>
+    </row>
+    <row r="344" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D344" t="s">
         <v>81</v>
       </c>
@@ -18841,7 +18849,7 @@
         <v>32.965395976923922</v>
       </c>
     </row>
-    <row r="345" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D345" t="s">
         <v>82</v>
       </c>
@@ -18904,7 +18912,7 @@
         <v>35.280224846589107</v>
       </c>
     </row>
-    <row r="346" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D346" t="s">
         <v>82</v>
       </c>
@@ -18967,7 +18975,7 @@
         <v>34.142153077344297</v>
       </c>
     </row>
-    <row r="347" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D347" t="s">
         <v>82</v>
       </c>
@@ -19030,7 +19038,7 @@
         <v>35.280224846589107</v>
       </c>
     </row>
-    <row r="348" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D348" t="s">
         <v>83</v>
       </c>
@@ -19093,7 +19101,7 @@
         <v>24.760247888708491</v>
       </c>
     </row>
-    <row r="349" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D349" t="s">
         <v>83</v>
       </c>
@@ -19156,7 +19164,7 @@
         <v>25.120396948907885</v>
       </c>
     </row>
-    <row r="350" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D350" t="s">
         <v>83</v>
       </c>
@@ -19219,7 +19227,7 @@
         <v>25.120396948907885</v>
       </c>
     </row>
-    <row r="351" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D351" t="s">
         <v>80</v>
       </c>
@@ -19278,14 +19286,14 @@
         <v>20</v>
       </c>
       <c r="X351" s="2">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Y351">
         <f>U351*V351*X351</f>
-        <v>38.914589377047619</v>
-      </c>
-    </row>
-    <row r="352" spans="1:25" x14ac:dyDescent="0.2">
+        <v>25.94305958469841</v>
+      </c>
+    </row>
+    <row r="352" spans="1:26" x14ac:dyDescent="0.2">
       <c r="D352" t="s">
         <v>80</v>
       </c>

</xml_diff>